<commit_message>
fixing some naming issues
</commit_message>
<xml_diff>
--- a/dm.xlsx
+++ b/dm.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2018-01-11</t>
+          <t>2011-01-18</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2018-01-12</t>
+          <t>2012-01-18</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2018-01-13</t>
+          <t>2013-01-18</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2017-12-31</t>
+          <t>2031-12-17</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2018-01-01</t>
+          <t>2001-01-18</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2018-01-02</t>
+          <t>2002-01-18</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2018-01-03</t>
+          <t>2003-01-18</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2018-01-13</t>
+          <t>2013-01-18</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2018-01-20</t>
+          <t>2020-01-18</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2018-01-16</t>
+          <t>2016-01-18</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2018-01-19</t>
+          <t>2019-01-18</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2018-01-22</t>
+          <t>2022-01-18</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2018-01-16</t>
+          <t>2016-01-18</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2018-01-21</t>
+          <t>2021-01-18</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2018-01-23</t>
+          <t>2023-01-18</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2018-01-05</t>
+          <t>2005-01-18</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2018-01-06</t>
+          <t>2006-01-18</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2018-01-16</t>
+          <t>2016-01-18</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2018-01-08</t>
+          <t>2008-01-18</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2018-01-20</t>
+          <t>2020-01-18</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2018-01-19</t>
+          <t>2019-01-18</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2018-01-23</t>
+          <t>2023-01-18</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2018-01-22</t>
+          <t>2022-01-18</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2018-01-23</t>
+          <t>2023-01-18</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2018-01-02</t>
+          <t>2002-01-18</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2018-01-17</t>
+          <t>2017-01-18</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2018-01-15</t>
+          <t>2015-01-18</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2018-01-14</t>
+          <t>2014-01-18</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2018-01-09</t>
+          <t>2009-01-18</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">

</xml_diff>

<commit_message>
fixing some sorting issues
</commit_message>
<xml_diff>
--- a/dm.xlsx
+++ b/dm.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PEAR1409151102-02092</t>
+          <t>PEAR14091511-BRZ02-02092</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>BRZ02</t>
         </is>
       </c>
       <c r="N2">
@@ -547,7 +547,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -555,9 +555,19 @@
           <t>PEAR14</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>BRZ</t>
+          <t>BRA</t>
         </is>
       </c>
     </row>
@@ -574,7 +584,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PEAR1409151102-02103</t>
+          <t>PEAR14091511-BRZ02-02103</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -599,7 +609,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>BRZ02</t>
         </is>
       </c>
       <c r="N3">
@@ -617,7 +627,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>AMERICAN INDIAN</t>
+          <t>AMERICAN INDIAN OR ALASKA NATIVE</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -627,7 +637,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -635,9 +645,19 @@
           <t>PLACEBO</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>BRZ</t>
+          <t>BRA</t>
         </is>
       </c>
     </row>
@@ -654,7 +674,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PEAR1409151103-05662</t>
+          <t>PEAR14091511-BRZ03-05662</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -679,7 +699,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>BRZ03</t>
         </is>
       </c>
       <c r="N4">
@@ -692,7 +712,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>UNDIFFERENTIATED</t>
+          <t>U</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -707,7 +727,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -715,9 +735,19 @@
           <t>PLACEBO</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>BRZ</t>
+          <t>BRA</t>
         </is>
       </c>
     </row>
@@ -734,7 +764,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PEAR1409151102-01001</t>
+          <t>PEAR14091511-CAN02-01001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -749,7 +779,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>CAN02</t>
         </is>
       </c>
       <c r="N5">
@@ -794,7 +824,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PEAR1409151102-01002</t>
+          <t>PEAR14091511-CAN02-01002</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -819,7 +849,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>CAN02</t>
         </is>
       </c>
       <c r="N6">
@@ -847,10 +877,20 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>PLACEBO</t>
         </is>
@@ -874,7 +914,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PEAR1409151107-01001</t>
+          <t>PEAR14091511-CAN07-01001</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -899,7 +939,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>CAN07</t>
         </is>
       </c>
       <c r="N7">
@@ -927,10 +967,20 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -954,7 +1004,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PEAR1409151109-01002</t>
+          <t>PEAR14091511-CAN09-01002</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -979,7 +1029,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>CAN09</t>
         </is>
       </c>
       <c r="N8">
@@ -1007,10 +1057,20 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -1034,7 +1094,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PEAR1409151105-90222</t>
+          <t>PEAR14091511-CHA05-90222</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1049,7 +1109,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>CHA05</t>
         </is>
       </c>
       <c r="N9">
@@ -1077,7 +1137,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CHN</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1154,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PEAR1409151105-90231</t>
+          <t>PEAR14091511-CHA05-90231</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1119,7 +1179,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>CHA05</t>
         </is>
       </c>
       <c r="N10">
@@ -1147,7 +1207,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1155,9 +1215,19 @@
           <t>PEAR14</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CHN</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1244,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PEAR1409151105-90902</t>
+          <t>PEAR14091511-CHA05-90902</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1189,7 +1259,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>CHA05</t>
         </is>
       </c>
       <c r="N11">
@@ -1217,7 +1287,7 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CHN</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1304,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PEAR1409151107-90630</t>
+          <t>PEAR14091511-CRO07-90630</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1259,7 +1329,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>CRO07</t>
         </is>
       </c>
       <c r="N12">
@@ -1287,7 +1357,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -1295,9 +1365,19 @@
           <t>PLACEBO</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>CRO</t>
+          <t>HRV</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1394,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PEAR1409151101-01021</t>
+          <t>PEAR14091511-CZE01-01021</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1339,7 +1419,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>CZE01</t>
         </is>
       </c>
       <c r="N13">
@@ -1367,10 +1447,20 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -1394,7 +1484,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PEAR1409151101-01011</t>
+          <t>PEAR14091511-DAN01-01011</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1419,7 +1509,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>DAN01</t>
         </is>
       </c>
       <c r="N14">
@@ -1447,7 +1537,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1455,9 +1545,19 @@
           <t>PEAR14</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>DAN</t>
+          <t>DNK</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1574,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PEAR1409151106-12112</t>
+          <t>PEAR14091511-EGP06-12112</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1489,7 +1589,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>EGP06</t>
         </is>
       </c>
       <c r="N15">
@@ -1507,7 +1607,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLACK OR AFRICAN AMERICAN</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1517,7 +1617,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>EGP</t>
+          <t>EGY</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1634,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PEAR1409151103-01002</t>
+          <t>PEAR14091511-ESP03-01002</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1559,7 +1659,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>ESP03</t>
         </is>
       </c>
       <c r="N16">
@@ -1587,10 +1687,20 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -1614,7 +1724,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PEAR1409151109-01007</t>
+          <t>PEAR14091511-ESP09-01007</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1639,7 +1749,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>ESP09</t>
         </is>
       </c>
       <c r="N17">
@@ -1667,10 +1777,20 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>PLACEBO</t>
         </is>
@@ -1694,7 +1814,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PEAR1409151106-01003</t>
+          <t>PEAR14091511-EST06-01003</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1719,7 +1839,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>EST06</t>
         </is>
       </c>
       <c r="N18">
@@ -1747,10 +1867,20 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
         <is>
           <t>PLACEBO</t>
         </is>
@@ -1774,7 +1904,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PEAR1409151109-01004</t>
+          <t>PEAR14091511-FRA09-01004</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1789,7 +1919,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>FRA09</t>
         </is>
       </c>
       <c r="N19">
@@ -1807,7 +1937,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>BLACK OR AFRICAN AMERICAN</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1834,7 +1964,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PEAR1409151129-02005</t>
+          <t>PEAR14091511-FRA29-02005</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1859,7 +1989,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>FRA29</t>
         </is>
       </c>
       <c r="N20">
@@ -1887,10 +2017,20 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -1914,7 +2054,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PEAR1409151101-97773</t>
+          <t>PEAR14091511-ISR01-97773</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1929,7 +2069,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>ISR01</t>
         </is>
       </c>
       <c r="N21">
@@ -1974,7 +2114,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PEAR1409151101-98974</t>
+          <t>PEAR14091511-ISR01-98974</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2004,7 +2144,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>ISR01</t>
         </is>
       </c>
       <c r="N22">
@@ -2032,10 +2172,20 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
         <is>
           <t>PLACEBO</t>
         </is>
@@ -2059,7 +2209,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PEAR1409151111-07851</t>
+          <t>PEAR14091511-ITL11-07851</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2084,7 +2234,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>ITL11</t>
         </is>
       </c>
       <c r="N23">
@@ -2112,7 +2262,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -2120,9 +2270,19 @@
           <t>PEAR14</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>ITA</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2299,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PEAR1409151111-09851</t>
+          <t>PEAR14091511-ITL11-09851</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2154,7 +2314,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>ITL11</t>
         </is>
       </c>
       <c r="N24">
@@ -2182,7 +2342,7 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>ITL</t>
+          <t>ITA</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2359,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PEAR1409151108-08031</t>
+          <t>PEAR14091511-JAP08-08031</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2214,7 +2374,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>JAP08</t>
         </is>
       </c>
       <c r="N25">
@@ -2242,7 +2402,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>JAP</t>
+          <t>JPN</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2419,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PEAR1409151101-08081</t>
+          <t>PEAR14091511-KOR01-08081</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2284,7 +2444,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>KOR01</t>
         </is>
       </c>
       <c r="N26">
@@ -2312,10 +2472,20 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
         <is>
           <t>PEAR14</t>
         </is>
@@ -2339,7 +2509,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PEAR1409151101-08093</t>
+          <t>PEAR14091511-KOR01-08093</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2354,7 +2524,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>KOR01</t>
         </is>
       </c>
       <c r="N27">
@@ -2399,7 +2569,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PEAR1409151108-07044</t>
+          <t>PEAR14091511-NOR08-07044</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2424,7 +2594,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>NOR08</t>
         </is>
       </c>
       <c r="N28">
@@ -2452,10 +2622,20 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
         <is>
           <t>PLACEBO</t>
         </is>
@@ -2479,7 +2659,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PEAR1409151109-80780</t>
+          <t>PEAR14091511-POR09-80780</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2494,7 +2674,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>POR09</t>
         </is>
       </c>
       <c r="N29">
@@ -2522,7 +2702,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>PRT</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2719,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PEAR1409151109-80891</t>
+          <t>PEAR14091511-POR09-80891</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2564,7 +2744,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>POR09</t>
         </is>
       </c>
       <c r="N30">
@@ -2592,7 +2772,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>PLCB</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -2600,9 +2780,19 @@
           <t>PLACEBO</t>
         </is>
       </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>PLCB</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>PLACEBO</t>
+        </is>
+      </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>PRT</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2809,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PEAR1409151111-11210</t>
+          <t>PEAR14091511-SLO11-11210</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2644,12 +2834,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>7-Feb-18</t>
+          <t>07-Feb-18</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>SLO11</t>
         </is>
       </c>
       <c r="N31">
@@ -2677,7 +2867,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>PR14</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -2685,9 +2875,19 @@
           <t>PEAR14</t>
         </is>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>PR14</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>PEAR14</t>
+        </is>
+      </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>SLO</t>
+          <t>SVN</t>
         </is>
       </c>
     </row>

</xml_diff>